<commit_message>
feat(flappy): 대시 충전 문턱 열(dash_charge_min_fall = 29 m/s)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#FlappyConfig.xlsx
+++ b/table/Datas/#FlappyConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,6 +517,11 @@
           <t>finish_brake</t>
         </is>
       </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>dash_charge_min_fall</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -619,6 +624,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -726,6 +736,11 @@
       <c r="T4" t="inlineStr">
         <is>
           <t>finish_brake</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>dash_charge_min_fall</t>
         </is>
       </c>
     </row>
@@ -786,6 +801,9 @@
       </c>
       <c r="T5" t="n">
         <v>3.4</v>
+      </c>
+      <c r="U5" t="n">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(flappy): 기류 값 3열 · Hologram 층(10) · 기류 필드 주입
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#FlappyConfig.xlsx
+++ b/table/Datas/#FlappyConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,6 +522,21 @@
           <t>dash_charge_min_fall</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>airflow_up_accel</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>airflow_rise_cap</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>shaft_gravity_mult</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -629,6 +644,21 @@
           <t>float</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -741,6 +771,21 @@
       <c r="U4" t="inlineStr">
         <is>
           <t>dash_charge_min_fall</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>airflow_up_accel</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>airflow_rise_cap</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>shaft_gravity_mult</t>
         </is>
       </c>
     </row>
@@ -804,6 +849,15 @@
       </c>
       <c r="U5" t="n">
         <v>23.2</v>
+      </c>
+      <c r="V5" t="n">
+        <v>30</v>
+      </c>
+      <c r="W5" t="n">
+        <v>12</v>
+      </c>
+      <c r="X5" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(flappy): 대시 0.48초 · 2.2배 — 카트 부스터 모양(원래 거리의 1.2배) Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#FlappyConfig.xlsx
+++ b/table/Datas/#FlappyConfig.xlsx
@@ -821,10 +821,10 @@
         <v>0.6</v>
       </c>
       <c r="L5" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="M5" t="n">
-        <v>0.8</v>
+        <v>0.48</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat(table): Flappy 원조 물리값 + body_length 열 추가
ForwardSpeed 4.5·FlapImpulse 10.125·Gravity 33.75·MaxFallSpeed 11.25로
교체하고, 누운 캡슐 길이를 담을 body_length(float, 그룹 비움) 열을
마지막에 추가했다(=1.28). body_radius·body_height 등 나머지는 그대로다.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/#FlappyConfig.xlsx
+++ b/table/Datas/#FlappyConfig.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,6 +537,11 @@
           <t>shaft_gravity_mult</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>body_length</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -659,6 +664,11 @@
           <t>float</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -786,6 +796,11 @@
       <c r="X4" t="inlineStr">
         <is>
           <t>shaft_gravity_mult</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>body_length</t>
         </is>
       </c>
     </row>
@@ -794,16 +809,16 @@
         <v>1</v>
       </c>
       <c r="C5" t="n">
-        <v>6.8</v>
+        <v>4.5</v>
       </c>
       <c r="D5" t="n">
-        <v>18.6</v>
+        <v>10.125</v>
       </c>
       <c r="E5" t="n">
-        <v>59</v>
+        <v>33.75</v>
       </c>
       <c r="F5" t="n">
-        <v>30</v>
+        <v>11.25</v>
       </c>
       <c r="G5" t="n">
         <v>0.45</v>
@@ -858,6 +873,9 @@
       </c>
       <c r="X5" t="n">
         <v>2</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>1.28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>